<commit_message>
updated logs added week 8 logs
</commit_message>
<xml_diff>
--- a/Research Logs/Matt/Matt Baker - Week 7 Research Log.xlsx
+++ b/Research Logs/Matt/Matt Baker - Week 7 Research Log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RecoveryAdmin\Documents\BHB-Capstone\Research Logs\Matt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69C2CC83-B9F7-4113-85BA-180279D708DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C16F8229-4453-4330-A687-91F87D73C0A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="2910" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Research template" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="104">
   <si>
     <t>Date</t>
   </si>
@@ -337,13 +337,68 @@
     <t>https://www.sciencedirect.com/science/article/pii/S0950705125005490</t>
   </si>
   <si>
-    <t>Looking for ways digital forensics experts validate tool outputs and determine reliability</t>
-  </si>
-  <si>
-    <t>Google Scholar</t>
-  </si>
-  <si>
     <t>Found a good science direct source that I can use to help explain our problem, also offers a good description of the "RAG" approach to data retrieval solutions for LLMs, it is a concept that has shown up a lot so it presents a potential future research topic.</t>
+  </si>
+  <si>
+    <t>https://dl.acm.org/doi/10.2753/MIS0742-1222240302</t>
+  </si>
+  <si>
+    <t>Finding out more about design science in order to apply it to our project and work with Bryce using some of his highlighted sources.</t>
+  </si>
+  <si>
+    <t>https://publikationen.bibliothek.kit.edu/1000055012</t>
+  </si>
+  <si>
+    <t>This source gives good definitions on the key parts of DS including how to define artifacts, what the 6 DS "activities" are, and how they can be integrated into IS projects. I like this source as it contained actual case study examples. I did not read the whole thing but it was a solid source of practical IS application os DS</t>
+  </si>
+  <si>
+    <t>This one gave a good history of DS and how it got revived and adapted into IS. Some of the graphs and sections especially the "state of the art" one were extremely hard for me to understand. The artefacts section was nice and gave a good definition an IS DSR artifact as a "tangible socio-technological instance in a DSR project which can
+be experienced, discussed, tested, evaluated, changed, improved, extended"</t>
+  </si>
+  <si>
+    <t>Understanding WinSCP and how it works</t>
+  </si>
+  <si>
+    <t>Reading/watching</t>
+  </si>
+  <si>
+    <t>I got a good understanding on what services need to be set up to get it to work and it should allow me to insert and retrieve our case files, 
+reports, and manage the directories inside of our remote desktop PC via FTP protocol</t>
+  </si>
+  <si>
+    <t>WinSCP documentation
+https://winscp.net/eng/docs/guides
+Tutorial
+https://www.youtube.com/watch?v=vtfpzSdlcGM</t>
+  </si>
+  <si>
+    <t>How to have a model inspect images with Ollama</t>
+  </si>
+  <si>
+    <t>https://docs.ollama.com/capabilities/vision</t>
+  </si>
+  <si>
+    <t>Provided the model and commands to present and give context to images within ollama. Only "vision" models have this capacity.</t>
+  </si>
+  <si>
+    <t>Collecting sources to read to try and find some information on prompt engineering in the digital forensics space</t>
+  </si>
+  <si>
+    <t>https://www.sciencedirect.com/science/article/pii/S2666281725001830</t>
+  </si>
+  <si>
+    <t>Looking for discussion/solutions on integration and prompt engineering challenges, specifically handling/processing data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exploring the potential of large language models for author profiling tasks in digital text forensics
+https://www.sciencedirect.com/science/article/pii/S2666281724001380?via%3Dihub
+</t>
+  </si>
+  <si>
+    <t>Found a couple of good ones to the topics im interested in, but most of them were blocked from access.</t>
+  </si>
+  <si>
+    <t>Interesting information and study about identifying individuals via their speech patterns, and from other languages. The "fine tuning strategies" for LLM inputes turned out not to be applicable insights for my project.</t>
   </si>
 </sst>
 </file>
@@ -353,7 +408,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d/mm/yy;@"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -373,6 +428,12 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -405,7 +466,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -422,6 +483,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -703,7 +767,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:G37"/>
+  <dimension ref="B2:G42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="13.140625" style="3" customWidth="1"/>
@@ -720,7 +784,7 @@
       </c>
       <c r="D2" s="5">
         <f>ROUNDDOWN(SUM(C6:C499)/60,0)</f>
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="E2" t="s">
         <v>8</v>
@@ -732,7 +796,7 @@
       </c>
       <c r="D3" s="5">
         <f>ROUND(MOD(SUM(C6:C499),60),0)</f>
-        <v>30</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.25">
@@ -1232,27 +1296,130 @@
         <v>83</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="G36" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="37" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:7" ht="90" x14ac:dyDescent="0.25">
       <c r="B37" s="3">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="C37">
-        <v>15</v>
+        <v>75</v>
       </c>
       <c r="D37" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>89</v>
       </c>
       <c r="G37" t="s">
         <v>86</v>
+      </c>
+    </row>
+    <row r="38" spans="2:7" ht="120" x14ac:dyDescent="0.25">
+      <c r="B38" s="3">
+        <v>46262</v>
+      </c>
+      <c r="C38">
+        <v>90</v>
+      </c>
+      <c r="D38" t="s">
+        <v>14</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="F38" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="39" spans="2:7" ht="75" x14ac:dyDescent="0.25">
+      <c r="B39" s="3">
+        <v>46263</v>
+      </c>
+      <c r="C39">
+        <v>30</v>
+      </c>
+      <c r="D39" t="s">
+        <v>92</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="G39" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="40" spans="2:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="B40" s="3">
+        <v>46264</v>
+      </c>
+      <c r="C40">
+        <v>15</v>
+      </c>
+      <c r="D40" t="s">
+        <v>14</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="41" spans="2:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="B41" s="3">
+        <v>46264</v>
+      </c>
+      <c r="C41">
+        <v>15</v>
+      </c>
+      <c r="D41" t="s">
+        <v>12</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="42" spans="2:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="B42" s="3">
+        <v>46264</v>
+      </c>
+      <c r="C42">
+        <v>60</v>
+      </c>
+      <c r="D42" t="s">
+        <v>14</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="G42" s="1" t="s">
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -1268,6 +1435,9 @@
     <hyperlink ref="G21" r:id="rId9" xr:uid="{7522D3CD-20E2-4229-AF82-ACF1397A1B5B}"/>
     <hyperlink ref="G22" r:id="rId10" xr:uid="{DBCF171A-04D2-44D4-A2C5-2BE4906AC74E}"/>
     <hyperlink ref="G33" r:id="rId11" xr:uid="{CF18B84E-B962-4B60-95A4-36586E83537F}"/>
+    <hyperlink ref="G38" r:id="rId12" xr:uid="{D3480BE9-0589-4FBC-A0E0-13FB89413A66}"/>
+    <hyperlink ref="G40" r:id="rId13" xr:uid="{2262C66A-11D9-4793-BA3D-07ECED0094C3}"/>
+    <hyperlink ref="G41" r:id="rId14" xr:uid="{6D648B93-C8C2-4BA9-B5BE-901807FAB9A4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>